<commit_message>
limpie SV, concatenar homogenizar y numex limpia
</commit_message>
<xml_diff>
--- a/Selva Viva/celulosa_bulk_final.xlsx
+++ b/Selva Viva/celulosa_bulk_final.xlsx
@@ -8614,52 +8614,58 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>2147</v>
+        <v>2146</v>
       </c>
       <c r="B91" t="n">
-        <v>8889</v>
+        <v>8865</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Euphorbiaceae</t>
+          <t>Violaceae</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Pseudosenefeldera</t>
+          <t>Leonia</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>inclinata</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr"/>
+          <t>glycycarpa</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>3928</t>
+        </is>
+      </c>
       <c r="G91" t="n">
         <v>68</v>
       </c>
       <c r="H91" t="n">
         <v>2025</v>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="n">
+        <v>9865</v>
+      </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="n">
-        <v>41.9886199891232</v>
+        <v>50.7386705764376</v>
       </c>
       <c r="L91" t="n">
-        <v>-30.4633399452444</v>
+        <v>-32.9258451761764</v>
       </c>
       <c r="M91" t="n">
-        <v>0.024841004</v>
+        <v>0.02234992814914083</v>
       </c>
       <c r="N91" t="n">
-        <v>0.404913041</v>
+        <v>0.4489033340843991</v>
       </c>
       <c r="O91" t="n">
-        <v>1.312047979797978</v>
+        <v>2.108676665915091</v>
       </c>
       <c r="P91" t="n">
-        <v>-31.78777476139979</v>
+        <v>-33.46661356502295</v>
       </c>
       <c r="Q91" t="b">
         <v>0</v>
@@ -8683,7 +8689,7 @@
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>p68-8889</t>
+          <t>p68-8865</t>
         </is>
       </c>
       <c r="X91" t="inlineStr">
@@ -8691,40 +8697,32 @@
           <t>leaf pulverized</t>
         </is>
       </c>
-      <c r="Y91" t="inlineStr">
-        <is>
-          <t>p68-8889</t>
-        </is>
-      </c>
+      <c r="Y91" t="inlineStr"/>
       <c r="Z91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>2148</v>
+        <v>2147</v>
       </c>
       <c r="B92" t="n">
-        <v>8888</v>
+        <v>8889</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Simaroubaceae</t>
+          <t>Euphorbiaceae</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Simaba</t>
+          <t>Pseudosenefeldera</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>polyphylla</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>3929</t>
-        </is>
-      </c>
+          <t>inclinata</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
         <v>68</v>
       </c>
@@ -8734,22 +8732,22 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="n">
-        <v>45.0545859187322</v>
+        <v>41.9886199891232</v>
       </c>
       <c r="L92" t="n">
-        <v>-33.0441162369113</v>
+        <v>-30.4633399452444</v>
       </c>
       <c r="M92" t="n">
-        <v>0.011420399</v>
+        <v>0.024841004</v>
       </c>
       <c r="N92" t="n">
-        <v>0.430948024</v>
+        <v>0.404913041</v>
       </c>
       <c r="O92" t="n">
-        <v>2.435300505050503</v>
+        <v>1.312047979797978</v>
       </c>
       <c r="P92" t="n">
-        <v>-34.86093531283139</v>
+        <v>-31.78777476139979</v>
       </c>
       <c r="Q92" t="b">
         <v>0</v>
@@ -8773,7 +8771,7 @@
       </c>
       <c r="W92" t="inlineStr">
         <is>
-          <t>p68-8888</t>
+          <t>p68-8889</t>
         </is>
       </c>
       <c r="X92" t="inlineStr">
@@ -8783,36 +8781,36 @@
       </c>
       <c r="Y92" t="inlineStr">
         <is>
-          <t>p68-8888</t>
+          <t>p68-8889</t>
         </is>
       </c>
       <c r="Z92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>2154</v>
+        <v>2148</v>
       </c>
       <c r="B93" t="n">
-        <v>8885</v>
+        <v>8888</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Apocynaceae</t>
+          <t>Simaroubaceae</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Aspidosperma</t>
+          <t>Simaba</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>aff. excelsum</t>
+          <t>polyphylla</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>3921</t>
+          <t>3929</t>
         </is>
       </c>
       <c r="G93" t="n">
@@ -8823,22 +8821,26 @@
       </c>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
+      <c r="K93" t="n">
+        <v>45.0545859187322</v>
+      </c>
+      <c r="L93" t="n">
+        <v>-33.0441162369113</v>
+      </c>
       <c r="M93" t="n">
-        <v>0.015294916</v>
+        <v>0.011420399</v>
       </c>
       <c r="N93" t="n">
-        <v>0.488282508</v>
+        <v>0.430948024</v>
       </c>
       <c r="O93" t="n">
-        <v>0.8692272727272705</v>
+        <v>2.435300505050503</v>
       </c>
       <c r="P93" t="n">
-        <v>-33.91217433722163</v>
+        <v>-34.86093531283139</v>
       </c>
       <c r="Q93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R93" t="b">
         <v>0</v>
@@ -8854,12 +8856,12 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>pesar celulosa</t>
+          <t>completo</t>
         </is>
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>p68-8885</t>
+          <t>p68-8888</t>
         </is>
       </c>
       <c r="X93" t="inlineStr">
@@ -8869,152 +8871,172 @@
       </c>
       <c r="Y93" t="inlineStr">
         <is>
-          <t>p68-8885</t>
+          <t>p68-8888</t>
         </is>
       </c>
       <c r="Z93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
+        <v>2154</v>
+      </c>
+      <c r="B94" t="n">
+        <v>8885</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Apocynaceae</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Aspidosperma</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>aff. excelsum</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>3921</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>68</v>
+      </c>
+      <c r="H94" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="n">
+        <v>0.015294916</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0.488282508</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.8692272727272705</v>
+      </c>
+      <c r="P94" t="n">
+        <v>-33.91217433722163</v>
+      </c>
+      <c r="Q94" t="b">
+        <v>1</v>
+      </c>
+      <c r="R94" t="b">
+        <v>0</v>
+      </c>
+      <c r="S94" t="b">
+        <v>0</v>
+      </c>
+      <c r="T94" t="b">
+        <v>0</v>
+      </c>
+      <c r="U94" t="b">
+        <v>0</v>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>pesar celulosa</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>p68-8885</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>leaf pulverized</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>p68-8885</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
         <v>2155</v>
       </c>
-      <c r="B94" t="n">
+      <c r="B95" t="n">
         <v>8883</v>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Melastomataceae</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>Miconia</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>sp</t>
         </is>
       </c>
-      <c r="F94">
+      <c r="F95">
         <f>3899</f>
         <v/>
       </c>
-      <c r="G94" t="n">
-        <v>68</v>
-      </c>
-      <c r="H94" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="n">
-        <v>40.9764178729058</v>
-      </c>
-      <c r="L94" t="n">
-        <v>-30.0244515471261</v>
-      </c>
-      <c r="M94" t="n">
-        <v>0.014952077</v>
-      </c>
-      <c r="N94" t="n">
-        <v>0.406260288</v>
-      </c>
-      <c r="O94" t="n">
-        <v>2.392098484848483</v>
-      </c>
-      <c r="P94" t="n">
-        <v>-31.90121357370095</v>
-      </c>
-      <c r="Q94" t="b">
-        <v>0</v>
-      </c>
-      <c r="R94" t="b">
-        <v>0</v>
-      </c>
-      <c r="S94" t="b">
-        <v>0</v>
-      </c>
-      <c r="T94" t="b">
-        <v>0</v>
-      </c>
-      <c r="U94" t="b">
-        <v>0</v>
-      </c>
-      <c r="V94" t="inlineStr">
-        <is>
-          <t>completo</t>
-        </is>
-      </c>
-      <c r="W94" t="inlineStr">
-        <is>
-          <t>p68-8883</t>
-        </is>
-      </c>
-      <c r="X94" t="inlineStr">
-        <is>
-          <t>leaf pulverized</t>
-        </is>
-      </c>
-      <c r="Y94" t="inlineStr">
-        <is>
-          <t>p68-8883</t>
-        </is>
-      </c>
-      <c r="Z94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr"/>
-      <c r="B95" t="n">
-        <v>8640</v>
-      </c>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="n">
         <v>68</v>
       </c>
       <c r="H95" t="n">
         <v>2025</v>
       </c>
-      <c r="I95" t="n">
-        <v>8640</v>
-      </c>
+      <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="n">
-        <v>44.8257164326167</v>
+        <v>40.9764178729058</v>
       </c>
       <c r="L95" t="n">
-        <v>-27.3770370113265</v>
-      </c>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
+        <v>-30.0244515471261</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0.014952077</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0.406260288</v>
+      </c>
+      <c r="O95" t="n">
+        <v>2.392098484848483</v>
+      </c>
+      <c r="P95" t="n">
+        <v>-31.90121357370095</v>
+      </c>
       <c r="Q95" t="b">
         <v>0</v>
       </c>
       <c r="R95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S95" t="b">
         <v>0</v>
       </c>
       <c r="T95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>pesar bulk; falta familia</t>
+          <t>completo</t>
         </is>
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>p68-8640</t>
+          <t>p68-8883</t>
         </is>
       </c>
       <c r="X95" t="inlineStr">
@@ -9022,13 +9044,17 @@
           <t>leaf pulverized</t>
         </is>
       </c>
-      <c r="Y95" t="inlineStr"/>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>p68-8883</t>
+        </is>
+      </c>
       <c r="Z95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="n">
-        <v>8865</v>
+        <v>8640</v>
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr"/>
@@ -9041,32 +9067,24 @@
         <v>2025</v>
       </c>
       <c r="I96" t="n">
-        <v>9865</v>
+        <v>8640</v>
       </c>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="n">
-        <v>50.7386705764376</v>
+        <v>44.8257164326167</v>
       </c>
       <c r="L96" t="n">
-        <v>-32.9258451761764</v>
-      </c>
-      <c r="M96" t="n">
-        <v>0.02234992814914083</v>
-      </c>
-      <c r="N96" t="n">
-        <v>0.4489033340843991</v>
-      </c>
-      <c r="O96" t="n">
-        <v>2.108676665915091</v>
-      </c>
-      <c r="P96" t="n">
-        <v>-33.46661356502295</v>
-      </c>
+        <v>-27.3770370113265</v>
+      </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
+      <c r="P96" t="inlineStr"/>
       <c r="Q96" t="b">
         <v>0</v>
       </c>
       <c r="R96" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S96" t="b">
         <v>0</v>
@@ -9079,12 +9097,12 @@
       </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>falta familia</t>
+          <t>pesar bulk; falta familia</t>
         </is>
       </c>
       <c r="W96" t="inlineStr">
         <is>
-          <t>p68-8865</t>
+          <t>p68-8640</t>
         </is>
       </c>
       <c r="X96" t="inlineStr">
@@ -13678,7 +13696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z32"/>
+  <dimension ref="A1:Z31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16062,63 +16080,61 @@
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>8865</v>
-      </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+        <v>3645</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Salicacia</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Laetia</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H29" t="n">
         <v>2025</v>
       </c>
-      <c r="I29" t="n">
-        <v>9865</v>
-      </c>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="n">
-        <v>50.7386705764376</v>
+        <v>42.6221781327326</v>
       </c>
       <c r="L29" t="n">
-        <v>-32.9258451761764</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0.02234992814914083</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0.4489033340843991</v>
-      </c>
-      <c r="O29" t="n">
-        <v>2.108676665915091</v>
-      </c>
-      <c r="P29" t="n">
-        <v>-33.46661356502295</v>
-      </c>
+        <v>-33.053099414117</v>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="b">
         <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" t="b">
         <v>0</v>
       </c>
       <c r="T29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U29" t="b">
         <v>1</v>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>falta familia</t>
+          <t>pesar bulk</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>p68-8865</t>
+          <t>p70-3645</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
@@ -16132,18 +16148,14 @@
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>3645</v>
+        <v>3650</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Salicacia</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Laetia</t>
-        </is>
-      </c>
+          <t>indet</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
@@ -16155,10 +16167,10 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>42.6221781327326</v>
+        <v>42.13</v>
       </c>
       <c r="L30" t="n">
-        <v>-33.053099414117</v>
+        <v>-31.61</v>
       </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
@@ -16186,7 +16198,7 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>p70-3645</t>
+          <t>p70-3650</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
@@ -16198,20 +16210,32 @@
       <c r="Z30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="n">
+        <v>2393</v>
+      </c>
       <c r="B31" t="n">
-        <v>3650</v>
+        <v>8832</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>indet</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+          <t>Violaceae</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Leonia</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>longifolium</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3270</v>
+      </c>
       <c r="G31" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H31" t="n">
         <v>2025</v>
@@ -16219,10 +16243,10 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="n">
-        <v>42.13</v>
+        <v>40.509559197114</v>
       </c>
       <c r="L31" t="n">
-        <v>-31.61</v>
+        <v>-32.1358652529169</v>
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
@@ -16241,7 +16265,7 @@
         <v>0</v>
       </c>
       <c r="U31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V31" t="inlineStr">
         <is>
@@ -16250,7 +16274,7 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>p70-3650</t>
+          <t>p74-8832</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
@@ -16260,82 +16284,6 @@
       </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>2393</v>
-      </c>
-      <c r="B32" t="n">
-        <v>8832</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Violaceae</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Leonia</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>longifolium</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>3270</v>
-      </c>
-      <c r="G32" t="n">
-        <v>74</v>
-      </c>
-      <c r="H32" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="n">
-        <v>40.509559197114</v>
-      </c>
-      <c r="L32" t="n">
-        <v>-32.1358652529169</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="b">
-        <v>0</v>
-      </c>
-      <c r="R32" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" t="b">
-        <v>0</v>
-      </c>
-      <c r="T32" t="b">
-        <v>0</v>
-      </c>
-      <c r="U32" t="b">
-        <v>0</v>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>pesar bulk</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>p74-8832</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>leaf pulverized</t>
-        </is>
-      </c>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16443,10 +16391,10 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>